<commit_message>
[auto-snapshot] 2026-04-15 12:00 | onda-hompage | 32 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_derma/남구_피부과.xlsx
+++ b/naver-place-crawler/results_derma/남구_피부과.xlsx
@@ -624,10 +624,10 @@
         <v>3632</v>
       </c>
       <c r="Q2" t="n">
-        <v>9994</v>
+        <v>9995</v>
       </c>
       <c r="R2" t="n">
-        <v>13626</v>
+        <v>13627</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -685,12 +685,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -706,12 +706,12 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P3" t="n">
@@ -906,10 +906,10 @@
         <v>1434</v>
       </c>
       <c r="Q5" t="n">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="R5" t="n">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -943,11 +943,7 @@
           <t>마리의원</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>marines8385@naver.com</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
@@ -1094,10 +1090,10 @@
         <v>272</v>
       </c>
       <c r="Q7" t="n">
-        <v>1349</v>
+        <v>1351</v>
       </c>
       <c r="R7" t="n">
-        <v>1621</v>
+        <v>1623</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1155,7 +1151,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1319,7 +1315,11 @@
           <t>문피부과의원</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>de_calcomani@naver.com</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
@@ -1414,11 +1414,7 @@
           <t>re-ele@naver.com</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>webtick@gmail.com</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>1644-2638</t>
@@ -1437,7 +1433,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1470,10 +1466,10 @@
         <v>2230</v>
       </c>
       <c r="Q11" t="n">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="R11" t="n">
-        <v>2989</v>
+        <v>2991</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1561,13 +1557,13 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Q12" t="n">
         <v>74</v>
       </c>
       <c r="R12" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1695,11 +1691,7 @@
           <t>세란피부과의원</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>lllllhope@naver.com</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
@@ -1903,7 +1895,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1973,11 +1965,7 @@
           <t>리앤리의원</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>inme2022@naver.com</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
@@ -2255,7 +2243,11 @@
           <t>리버스의원 인천구월 터미널역</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>wlskfl9087@naver.com</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
@@ -2280,7 +2272,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2308,10 +2300,10 @@
         <v>632</v>
       </c>
       <c r="Q20" t="n">
-        <v>2178</v>
+        <v>2177</v>
       </c>
       <c r="R20" t="n">
-        <v>2810</v>
+        <v>2809</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
@@ -2496,10 +2488,10 @@
         <v>1858</v>
       </c>
       <c r="Q22" t="n">
-        <v>6814</v>
+        <v>6818</v>
       </c>
       <c r="R22" t="n">
-        <v>8672</v>
+        <v>8676</v>
       </c>
       <c r="S22" t="inlineStr">
         <is>
@@ -2815,11 +2807,7 @@
           <t>인천CNP차앤박피부과</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>cnpskin07@naver.com</t>
-        </is>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
@@ -2844,7 +2832,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -3191,11 +3179,7 @@
           <t>장피부과의원</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>1sanginfl@naver.com</t>
-        </is>
-      </c>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>jangskin@lycos.co.kr</t>
@@ -3289,7 +3273,11 @@
           <t>이지피부과</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>towhsb@naver.com</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
@@ -3501,12 +3489,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3595,7 +3583,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -3722,10 +3710,10 @@
         <v>248</v>
       </c>
       <c r="Q35" t="n">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="R35" t="n">
-        <v>363</v>
+        <v>342</v>
       </c>
       <c r="S35" t="inlineStr">
         <is>
@@ -3855,7 +3843,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>limka0917@naver.com</t>
+          <t>social_forum@naver.com</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -4102,10 +4090,10 @@
         <v>9367</v>
       </c>
       <c r="Q39" t="n">
-        <v>2378</v>
+        <v>2393</v>
       </c>
       <c r="R39" t="n">
-        <v>11745</v>
+        <v>11760</v>
       </c>
       <c r="S39" t="inlineStr">
         <is>
@@ -4327,11 +4315,7 @@
           <t>맑고고운의원 옥련송도역점</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>value_trend_guide@naver.com</t>
-        </is>
-      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
@@ -4666,10 +4650,10 @@
         <v>43</v>
       </c>
       <c r="Q45" t="n">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="R45" t="n">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="S45" t="inlineStr">
         <is>
@@ -5504,10 +5488,10 @@
         <v>5244</v>
       </c>
       <c r="Q54" t="n">
-        <v>3927</v>
+        <v>3935</v>
       </c>
       <c r="R54" t="n">
-        <v>9171</v>
+        <v>9179</v>
       </c>
       <c r="S54" t="inlineStr">
         <is>
@@ -5565,12 +5549,12 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -5659,7 +5643,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -5692,10 +5676,10 @@
         <v>1516</v>
       </c>
       <c r="Q56" t="n">
-        <v>5069</v>
+        <v>5070</v>
       </c>
       <c r="R56" t="n">
-        <v>6585</v>
+        <v>6586</v>
       </c>
       <c r="S56" t="inlineStr">
         <is>
@@ -6105,7 +6089,11 @@
           <t>주안연세의원</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>lan_j_97@naver.com</t>
+        </is>
+      </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
@@ -6289,11 +6277,7 @@
           <t>봄헤어뷰티살롱</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>yallycry@naver.com</t>
-        </is>
-      </c>
+      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
@@ -6665,11 +6649,7 @@
           <t>한상희비뇨기과의원</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>yurim2224@naver.com</t>
-        </is>
-      </c>
+      <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
@@ -6759,7 +6739,11 @@
           <t>인하비뇨기과의원</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>binterest@naver.com</t>
+        </is>
+      </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
@@ -6784,7 +6768,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -6849,11 +6833,7 @@
           <t>이인의비뇨기과의원</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>binterest@naver.com</t>
-        </is>
-      </c>
+      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
@@ -6943,11 +6923,7 @@
           <t>W여성병원</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>jeilwomen@naver.com</t>
-        </is>
-      </c>
+      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
@@ -7000,10 +6976,10 @@
         <v>6165</v>
       </c>
       <c r="Q70" t="n">
-        <v>2166</v>
+        <v>2167</v>
       </c>
       <c r="R70" t="n">
-        <v>8331</v>
+        <v>8332</v>
       </c>
       <c r="S70" t="inlineStr">
         <is>
@@ -7070,7 +7046,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -7135,7 +7111,11 @@
           <t>쑥쑥튼튼소아청소년과의원</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>tteumodo@naver.com</t>
+        </is>
+      </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
@@ -7470,10 +7450,10 @@
         <v>1126</v>
       </c>
       <c r="Q75" t="n">
-        <v>5322</v>
+        <v>5324</v>
       </c>
       <c r="R75" t="n">
-        <v>6448</v>
+        <v>6450</v>
       </c>
       <c r="S75" t="inlineStr">
         <is>

</xml_diff>